<commit_message>
Mise à jour du tableau de synthèse pour le projet BTS
</commit_message>
<xml_diff>
--- a/public/tableau-synthese-bts-adrien-clavreul.xlsx
+++ b/public/tableau-synthese-bts-adrien-clavreul.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="40">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -168,6 +168,16 @@
   </si>
   <si>
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serveur Debian, Docker &amp; déploiement continu — CNFPT Rennes
+  › Rapports d'audit OpenSCAP (43 % → 91 %) et scripts de remédiation
+  › Stacks Docker déployées via Portainer depuis Gitea (CI/CD)
+  › Reverse proxy Nginx Proxy Manager avec SSL automatique
+  › Sauvegardes quotidiennes des volumes et BDD vers un NAS</t>
+  </si>
+  <si>
+    <t>07/26 → 12/26</t>
   </si>
 </sst>
 </file>
@@ -1531,14 +1541,30 @@
       <c r="H27" s="35"/>
     </row>
     <row r="28" ht="75" customHeight="1" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="29"/>
-      <c r="B28" s="30"/>
-      <c r="C28" s="31"/>
-      <c r="D28" s="31"/>
-      <c r="E28" s="31"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="31"/>
-      <c r="H28" s="32"/>
+      <c r="A28" s="29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D28" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="E28" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="F28" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="H28" s="32" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="29" ht="39.95" customHeight="1" spans="1:8" s="21" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="29"/>

</xml_diff>